<commit_message>
feat: add RecipeDetailScreen component for displaying recipe details, including ingredients, steps, and favorite functionality
</commit_message>
<xml_diff>
--- a/api.xlsx
+++ b/api.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Ki6\Lap trinh ung ung di dong\pro\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D483A02-FC18-43C1-8DFC-4992D2829172}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DDD5FDB-D2B1-41D6-BD36-949CAEC34086}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1515" yWindow="1515" windowWidth="21600" windowHeight="12645" xr2:uid="{33F52725-B95F-4C8F-9B17-586DBC465F5D}"/>
+    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="17385" xr2:uid="{33F52725-B95F-4C8F-9B17-586DBC465F5D}"/>
   </bookViews>
   <sheets>
     <sheet name="Trang_tính1" sheetId="1" r:id="rId1"/>
@@ -36,25 +36,37 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>URL</t>
   </si>
   <si>
-    <t>MÔ TẢ</t>
+    <t>METHOD</t>
   </si>
   <si>
-    <t>CHỨC NĂNG</t>
+    <t> http://localhost:3000/api/auth/login</t>
   </si>
   <si>
-    <t>KẾT QUẢ</t>
+    <t>POST</t>
+  </si>
+  <si>
+    <t>Body</t>
+  </si>
+  <si>
+    <t>Trả về</t>
+  </si>
+  <si>
+    <t>Mô tả chức năng</t>
+  </si>
+  <si>
+    <t>…</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -63,6 +75,30 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="15"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
@@ -70,7 +106,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -80,6 +116,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="4" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -108,18 +150,25 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Bình thường" xfId="0" builtinId="0"/>
+    <cellStyle name="Siêu kết nối" xfId="1" builtinId="8"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -451,150 +500,205 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{06AFDF30-2E97-4C2E-8BD7-ABFE4925599E}">
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24.5703125" customWidth="1"/>
-    <col min="2" max="2" width="34.5703125" customWidth="1"/>
+    <col min="2" max="2" width="53" customWidth="1"/>
     <col min="3" max="3" width="37.140625" customWidth="1"/>
     <col min="4" max="4" width="30.5703125" customWidth="1"/>
+    <col min="5" max="5" width="16.85546875" customWidth="1"/>
+    <col min="6" max="6" width="29.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="39" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:6" ht="39" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="1"/>
-      <c r="B2" s="1"/>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="1"/>
-      <c r="B3" s="1"/>
-      <c r="C3" s="1"/>
-      <c r="D3" s="1"/>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="1"/>
-      <c r="B4" s="1"/>
-      <c r="C4" s="1"/>
-      <c r="D4" s="1"/>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="1"/>
-      <c r="B5" s="1"/>
-      <c r="C5" s="1"/>
-      <c r="D5" s="1"/>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="1"/>
-      <c r="B6" s="1"/>
-      <c r="C6" s="1"/>
-      <c r="D6" s="1"/>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="1"/>
-      <c r="B7" s="1"/>
-      <c r="C7" s="1"/>
-      <c r="D7" s="1"/>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" s="1"/>
-      <c r="B8" s="1"/>
-      <c r="C8" s="1"/>
-      <c r="D8" s="1"/>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="1"/>
-      <c r="B9" s="1"/>
-      <c r="C9" s="1"/>
-      <c r="D9" s="1"/>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="1"/>
-      <c r="B10" s="1"/>
-      <c r="C10" s="1"/>
-      <c r="D10" s="1"/>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="1"/>
-      <c r="B11" s="1"/>
-      <c r="C11" s="1"/>
-      <c r="D11" s="1"/>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="1"/>
-      <c r="B12" s="1"/>
-      <c r="C12" s="1"/>
-      <c r="D12" s="1"/>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" s="1"/>
-      <c r="B13" s="1"/>
-      <c r="C13" s="1"/>
-      <c r="D13" s="1"/>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" s="1"/>
-      <c r="B14" s="1"/>
-      <c r="C14" s="1"/>
-      <c r="D14" s="1"/>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" s="1"/>
-      <c r="B15" s="1"/>
-      <c r="C15" s="1"/>
-      <c r="D15" s="1"/>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" s="1"/>
-      <c r="B16" s="1"/>
-      <c r="C16" s="1"/>
-      <c r="D16" s="1"/>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" s="1"/>
-      <c r="B17" s="1"/>
-      <c r="C17" s="1"/>
-      <c r="D17" s="1"/>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" s="1"/>
-      <c r="B18" s="1"/>
-      <c r="C18" s="1"/>
-      <c r="D18" s="1"/>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" s="1"/>
-      <c r="B19" s="1"/>
-      <c r="C19" s="1"/>
-      <c r="D19" s="1"/>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="1"/>
-      <c r="B20" s="1"/>
-      <c r="C20" s="1"/>
-      <c r="D20" s="1"/>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" s="1"/>
-      <c r="B21" s="1"/>
-      <c r="C21" s="1"/>
-      <c r="D21" s="1"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+    </row>
+    <row r="3" spans="1:6" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="A3" s="2"/>
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+    </row>
+    <row r="4" spans="1:6" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="A4" s="2"/>
+      <c r="B4" s="2"/>
+      <c r="C4" s="2"/>
+      <c r="D4" s="2"/>
+      <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
+    </row>
+    <row r="5" spans="1:6" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="A5" s="2"/>
+      <c r="B5" s="2"/>
+      <c r="C5" s="2"/>
+      <c r="D5" s="2"/>
+      <c r="E5" s="2"/>
+      <c r="F5" s="2"/>
+    </row>
+    <row r="6" spans="1:6" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="A6" s="2"/>
+      <c r="B6" s="2"/>
+      <c r="C6" s="2"/>
+      <c r="D6" s="2"/>
+      <c r="E6" s="2"/>
+      <c r="F6" s="2"/>
+    </row>
+    <row r="7" spans="1:6" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="A7" s="2"/>
+      <c r="B7" s="2"/>
+      <c r="C7" s="2"/>
+      <c r="D7" s="2"/>
+      <c r="E7" s="2"/>
+      <c r="F7" s="2"/>
+    </row>
+    <row r="8" spans="1:6" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="A8" s="2"/>
+      <c r="B8" s="2"/>
+      <c r="C8" s="2"/>
+      <c r="D8" s="2"/>
+      <c r="E8" s="2"/>
+      <c r="F8" s="2"/>
+    </row>
+    <row r="9" spans="1:6" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="A9" s="2"/>
+      <c r="B9" s="2"/>
+      <c r="C9" s="2"/>
+      <c r="D9" s="2"/>
+      <c r="E9" s="2"/>
+      <c r="F9" s="2"/>
+    </row>
+    <row r="10" spans="1:6" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="A10" s="2"/>
+      <c r="B10" s="2"/>
+      <c r="C10" s="2"/>
+      <c r="D10" s="2"/>
+      <c r="E10" s="2"/>
+      <c r="F10" s="2"/>
+    </row>
+    <row r="11" spans="1:6" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="A11" s="2"/>
+      <c r="B11" s="2"/>
+      <c r="C11" s="2"/>
+      <c r="D11" s="2"/>
+      <c r="E11" s="2"/>
+      <c r="F11" s="2"/>
+    </row>
+    <row r="12" spans="1:6" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="A12" s="2"/>
+      <c r="B12" s="2"/>
+      <c r="C12" s="2"/>
+      <c r="D12" s="2"/>
+      <c r="E12" s="2"/>
+      <c r="F12" s="2"/>
+    </row>
+    <row r="13" spans="1:6" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="A13" s="2"/>
+      <c r="B13" s="2"/>
+      <c r="C13" s="2"/>
+      <c r="D13" s="2"/>
+      <c r="E13" s="2"/>
+      <c r="F13" s="2"/>
+    </row>
+    <row r="14" spans="1:6" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="A14" s="2"/>
+      <c r="B14" s="2"/>
+      <c r="C14" s="2"/>
+      <c r="D14" s="2"/>
+      <c r="E14" s="2"/>
+      <c r="F14" s="2"/>
+    </row>
+    <row r="15" spans="1:6" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="A15" s="2"/>
+      <c r="B15" s="2"/>
+      <c r="C15" s="2"/>
+      <c r="D15" s="2"/>
+      <c r="E15" s="2"/>
+      <c r="F15" s="2"/>
+    </row>
+    <row r="16" spans="1:6" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="A16" s="2"/>
+      <c r="B16" s="2"/>
+      <c r="C16" s="2"/>
+      <c r="D16" s="2"/>
+      <c r="E16" s="2"/>
+      <c r="F16" s="2"/>
+    </row>
+    <row r="17" spans="1:6" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="A17" s="2"/>
+      <c r="B17" s="2"/>
+      <c r="C17" s="2"/>
+      <c r="D17" s="2"/>
+      <c r="E17" s="2"/>
+      <c r="F17" s="2"/>
+    </row>
+    <row r="18" spans="1:6" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="A18" s="2"/>
+      <c r="B18" s="2"/>
+      <c r="C18" s="2"/>
+      <c r="D18" s="2"/>
+      <c r="E18" s="2"/>
+      <c r="F18" s="2"/>
+    </row>
+    <row r="19" spans="1:6" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="A19" s="2"/>
+      <c r="B19" s="2"/>
+      <c r="C19" s="2"/>
+      <c r="D19" s="2"/>
+      <c r="E19" s="2"/>
+      <c r="F19" s="2"/>
+    </row>
+    <row r="20" spans="1:6" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="A20" s="2"/>
+      <c r="B20" s="2"/>
+      <c r="C20" s="2"/>
+      <c r="D20" s="2"/>
+      <c r="E20" s="2"/>
+      <c r="F20" s="2"/>
+    </row>
+    <row r="21" spans="1:6" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="A21" s="2"/>
+      <c r="B21" s="2"/>
+      <c r="C21" s="2"/>
+      <c r="D21" s="2"/>
+      <c r="E21" s="2"/>
+      <c r="F21" s="2"/>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B2" r:id="rId1" display="vscode-file://vscode-app/c:/Users/ADMIN/AppData/Local/Programs/Microsoft VS Code/ce099c1ed2/resources/app/out/vs/code/electron-browser/workbench/workbench.html" xr:uid="{48AE9BAA-EE24-4CB4-913E-6B0824093238}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>